<commit_message>
Testing Result is added
</commit_message>
<xml_diff>
--- a/output/inspection_report.xlsx
+++ b/output/inspection_report.xlsx
@@ -425,46 +425,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Inspection ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Date / Time</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Panel ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>RGB Finding</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>RGB Confidence</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Thermal Finding</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Thermal Confidence</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -473,306 +478,724 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>P001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>bird-drop, clean</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.08319041132926941</v>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Require Inspection</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>P002</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>P003</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>P004</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>P005</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>P006</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>P007</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>P008</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>23-09-2026 17:36:50</t>
+          <t>INS-001</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>P009</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>No Finding</t>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>P010</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>bird-drop, bird-drop</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1347211003303528</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Require Inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>P011</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>bird-drop, bird-drop</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0.1544758677482605</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Require Inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>P012</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>P013</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>bird-drop</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.08045026659965515</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Require Inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>P014</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>P015</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>P016</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>P017</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>P018</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>bird-drop</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0.05383062362670898</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Require Inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P019</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>bird-drop</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.05319708585739136</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Require Inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>P020</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>bird-drop</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.1283735930919647</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>RGB</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Require Inspection</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>P021</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>INS-001</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>25-09-2026 12:43:42</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>P022</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>No RGB Defect Detected</t>
         </is>
       </c>
     </row>

</xml_diff>